<commit_message>
Fix corrupted xlsx: patch chart XML with valid dual-axis structure
Co-authored-by: IBonsaiBob <217611143+IBonsaiBob@users.noreply.github.com>
Agent-Logs-Url: https://github.com/IBonsaiBob/flow-pressure-dashboard/sessions/34c92cf3-5df0-4c97-b8c6-a8f16b655547
</commit_message>
<xml_diff>
--- a/Flow_Pressure_Dashboard.xlsx
+++ b/Flow_Pressure_Dashboard.xlsx
@@ -423,162 +423,165 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
           <a:bodyPr/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
             <a:r>
               <a:t>Flow &amp; Pressure Analysis</a:t>
             </a:r>
           </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!C24</f>
-            </strRef>
-          </tx>
-          <spPr>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$24</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:ln w="20000">
               <a:solidFill>
                 <a:srgbClr val="2E75B6"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$25:$A$124</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$C$25:$C$124</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="100"/>
-      </lineChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!E24</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Dashboard!$A$25:$A$124</c:f>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$25:$C$124</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1001"/>
+        <c:axId val="1002"/>
+      </c:lineChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$E$24</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="C55A11"/>
+              </a:solidFill>
             </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$25:$A$124</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$E$25:$E$124</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="100"/>
-        <axId val="200"/>
-      </lineChart>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Dashboard!$A$25:$A$124</c:f>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$E$25:$E$124</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1001"/>
+        <c:axId val="1003"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="m/d/yy" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="1002"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
               <a:bodyPr/>
               <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
                 <a:r>
                   <a:t>Flow Adjusted</a:t>
                 </a:r>
               </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="r"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="1001"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1003"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
               <a:bodyPr/>
               <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
                 <a:r>
                   <a:t>Pressure Adjusted</a:t>
                 </a:r>
               </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crosses val="max"/>
+        <c:crossAx val="1001"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Fix xlsx: complete Excel-compatible chart XML and place [Content_Types].xml first in ZIP
- Add missing elements to chart XML that Excel requires: c:lang, c:layout,
  c:lstStyle, c:pPr/c:defRPr in text runs, c:smooth, c:tickLblPos,
  c:crosses/autoZero, c:crossBetween/between, c:showDLblsOverMax,
  c:overlay in legend, c:numFmt on value axes
- Fix _patch_chart_xml to write [Content_Types].xml as the first entry
  in the ZIP, as required by the OPC/OOXML specification
- Regenerate Flow_Pressure_Dashboard.xlsx

Co-authored-by: IBonsaiBob <217611143+IBonsaiBob@users.noreply.github.com>
Agent-Logs-Url: https://github.com/IBonsaiBob/flow-pressure-dashboard/sessions/754a6eb0-8978-49f1-a520-f9e08694f144
</commit_message>
<xml_diff>
--- a/Flow_Pressure_Dashboard.xlsx
+++ b/Flow_Pressure_Dashboard.xlsx
@@ -424,13 +424,18 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
   <c:style val="10"/>
   <c:chart>
     <c:title>
       <c:tx>
         <c:rich>
           <a:bodyPr/>
+          <a:lstStyle/>
           <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
             <a:r>
               <a:t>Flow &amp; Pressure Analysis</a:t>
             </a:r>
@@ -441,6 +446,7 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
+      <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -462,6 +468,7 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:smooth val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Dashboard!$A$25:$A$124</c:f>
@@ -473,6 +480,10 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:smooth val="0"/>
         <c:axId val="1001"/>
         <c:axId val="1002"/>
       </c:lineChart>
@@ -497,6 +508,7 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:smooth val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Dashboard!$A$25:$A$124</c:f>
@@ -508,6 +520,10 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:smooth val="0"/>
         <c:axId val="1001"/>
         <c:axId val="1003"/>
       </c:lineChart>
@@ -519,9 +535,14 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="m/d/yy" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1002"/>
+        <c:auto val="1"/>
+        <c:lblAlign val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="1002"/>
@@ -535,7 +556,11 @@
           <c:tx>
             <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
                 <a:r>
                   <a:t>Flow Adjusted</a:t>
                 </a:r>
@@ -544,9 +569,13 @@
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="1003"/>
@@ -560,7 +589,11 @@
           <c:tx>
             <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
                 <a:r>
                   <a:t>Pressure Adjusted</a:t>
                 </a:r>
@@ -569,17 +602,22 @@
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1001"/>
         <c:crosses val="max"/>
-        <c:crossAx val="1001"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
 </c:chartSpace>
 </file>

</xml_diff>

<commit_message>
Fix Excel "Removed Part: drawing1.xml" — chart never shows on open
Excel was discarding xl/drawings/drawing1.xml on every open because
openpyxl generates an invalid drawing anchor XML. Add two new builders
(_build_correct_drawing_xml / _build_correct_drawing_rels) and extend
_patch_chart_xml to replace those files alongside chart1.xml.

Bugs fixed in drawing1.xml:
1. All spreadsheetDrawing elements used default xmlns= namespace instead
   of required xdr: prefix
2. <graphicFrame> missing required macro="" attribute
3. <xfrm /> was self-closing/empty — needs <a:off> and <a:ext> children
4. Missing <?xml ...?> declaration

Bug fixed in drawing1.xml.rels:
5. Relationship Target was absolute /xl/charts/chart1.xml, changed to
   relative ../charts/chart1.xml

Co-authored-by: IBonsaiBob <217611143+IBonsaiBob@users.noreply.github.com>
Agent-Logs-Url: https://github.com/IBonsaiBob/flow-pressure-dashboard/sessions/a1720891-7277-4001-847a-7b4fc702a4ef
</commit_message>
<xml_diff>
--- a/Flow_Pressure_Dashboard.xlsx
+++ b/Flow_Pressure_Dashboard.xlsx
@@ -1219,30 +1219,33 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7200000" cy="5040000"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Re-enable drawing1.xml patch: fix missing required macro= on graphicFrame
Two OOXML compliance failures were both needed to fix the repair dialog:
1. c:smooth before c:cat/c:val in chart XML (fixed last session)
2. openpyxl omits required macro='' on <graphicFrame> (fixed this session)

_patch_chart_xml() now replaces chart1.xml + drawing1.xml + drawing rels

Co-authored-by: IBonsaiBob <217611143+IBonsaiBob@users.noreply.github.com>
Agent-Logs-Url: https://github.com/IBonsaiBob/flow-pressure-dashboard/sessions/6071beb5-99da-47b0-91e8-2e5d7b634ee6
</commit_message>
<xml_diff>
--- a/Flow_Pressure_Dashboard.xlsx
+++ b/Flow_Pressure_Dashboard.xlsx
@@ -1605,30 +1605,40 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>799200</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>112400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Fix CT_LineChart.marker type: remove invalid CT_Marker at lineChart level
CT_LineChart.marker is CT_Boolean (<c:marker val="0"/>), not CT_Marker
(<c:marker><c:symbol .../>). The complex element form was causing Excel to
reject chart1.xml and cascade-remove drawing1.xml (the repair dialog bug).

Co-authored-by: IBonsaiBob <217611143+IBonsaiBob@users.noreply.github.com>
Agent-Logs-Url: https://github.com/IBonsaiBob/flow-pressure-dashboard/sessions/e587a431-1b92-4725-8081-a38fc931ca5e
</commit_message>
<xml_diff>
--- a/Flow_Pressure_Dashboard.xlsx
+++ b/Flow_Pressure_Dashboard.xlsx
@@ -738,9 +738,6 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
         <c:smooth val="0"/>
         <c:axId val="1001"/>
         <c:axId val="1002"/>
@@ -1508,9 +1505,6 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
         <c:smooth val="0"/>
         <c:axId val="1001"/>
         <c:axId val="1003"/>

</xml_diff>